<commit_message>
qol: added projectile spread modifier (v1)
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5C3B131C-7D60-4310-84CD-058E223434D9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C049FD-EDA1-4BC9-9F51-E14FA9F3ED0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="85" uniqueCount="63">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -273,6 +273,18 @@
   </si>
   <si>
     <t>Deprecated</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ProjectileSpreadModifier</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>modify projectile (not the weapon) spread when firing a projectile</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>To modify projectile spread</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -317,7 +329,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="14">
+  <borders count="12">
     <border>
       <left/>
       <right/>
@@ -424,37 +436,13 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
       <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
@@ -464,10 +452,10 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
-        <color indexed="64"/>
-      </top>
-      <bottom/>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -500,34 +488,34 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="13" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -810,13 +798,13 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:H14"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="34.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="51" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="44.58203125" style="1" bestFit="1" customWidth="1"/>
     <col min="7" max="7" width="27.25" style="1" bestFit="1" customWidth="1"/>
@@ -831,13 +819,13 @@
       <c r="B1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="11" t="s">
+      <c r="C1" s="8" t="s">
         <v>17</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>18</v>
       </c>
-      <c r="E1" s="11" t="s">
+      <c r="E1" s="8" t="s">
         <v>19</v>
       </c>
       <c r="F1" s="7" t="s">
@@ -846,12 +834,12 @@
       <c r="G1" s="7" t="s">
         <v>21</v>
       </c>
-      <c r="H1" s="11" t="s">
+      <c r="H1" s="8" t="s">
         <v>53</v>
       </c>
     </row>
     <row r="2" spans="1:8">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="14" t="s">
         <v>13</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -877,7 +865,7 @@
       </c>
     </row>
     <row r="3" spans="1:8">
-      <c r="A3" s="13"/>
+      <c r="A3" s="15"/>
       <c r="B3" s="1" t="s">
         <v>48</v>
       </c>
@@ -901,7 +889,7 @@
       </c>
     </row>
     <row r="4" spans="1:8">
-      <c r="A4" s="13"/>
+      <c r="A4" s="15"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -923,23 +911,23 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8">
-      <c r="A5" s="14"/>
-      <c r="B5" s="15" t="s">
+      <c r="A5" s="16"/>
+      <c r="B5" s="10" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="15" t="s">
+      <c r="C5" s="10" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="15" t="s">
+      <c r="D5" s="10" t="s">
         <v>31</v>
       </c>
-      <c r="E5" s="15" t="s">
+      <c r="E5" s="10" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="15" t="s">
+      <c r="F5" s="10" t="s">
         <v>43</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="11" t="s">
         <v>10</v>
       </c>
       <c r="H5" s="4" t="s">
@@ -947,7 +935,7 @@
       </c>
     </row>
     <row r="6" spans="1:8">
-      <c r="A6" s="12" t="s">
+      <c r="A6" s="14" t="s">
         <v>15</v>
       </c>
       <c r="B6" s="2" t="s">
@@ -971,7 +959,7 @@
       <c r="H6" s="3"/>
     </row>
     <row r="7" spans="1:8">
-      <c r="A7" s="13"/>
+      <c r="A7" s="15"/>
       <c r="B7" s="1" t="s">
         <v>5</v>
       </c>
@@ -993,23 +981,23 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8">
-      <c r="A8" s="13"/>
-      <c r="B8" s="17" t="s">
+      <c r="A8" s="15"/>
+      <c r="B8" s="12" t="s">
         <v>6</v>
       </c>
-      <c r="C8" s="17" t="s">
+      <c r="C8" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="17" t="s">
+      <c r="D8" s="12" t="s">
         <v>32</v>
       </c>
-      <c r="E8" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="17" t="s">
+      <c r="E8" s="12" t="s">
+        <v>11</v>
+      </c>
+      <c r="F8" s="12" t="s">
         <v>43</v>
       </c>
-      <c r="G8" s="18" t="s">
+      <c r="G8" s="13" t="s">
         <v>2</v>
       </c>
       <c r="H8" s="4" t="s">
@@ -1017,7 +1005,7 @@
       </c>
     </row>
     <row r="9" spans="1:8">
-      <c r="A9" s="13"/>
+      <c r="A9" s="15"/>
       <c r="B9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1041,7 +1029,7 @@
       </c>
     </row>
     <row r="10" spans="1:8">
-      <c r="A10" s="13"/>
+      <c r="A10" s="15"/>
       <c r="B10" s="1" t="s">
         <v>9</v>
       </c>
@@ -1063,81 +1051,104 @@
       <c r="H10" s="4"/>
     </row>
     <row r="11" spans="1:8">
-      <c r="A11" s="14"/>
-      <c r="B11" s="5" t="s">
+      <c r="A11" s="15"/>
+      <c r="B11" s="17" t="s">
         <v>8</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="17" t="s">
         <v>28</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="17" t="s">
         <v>35</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="6" t="b">
+      <c r="E11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="F11" s="17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" s="4" t="b">
         <v>1</v>
       </c>
       <c r="H11" s="4"/>
     </row>
     <row r="12" spans="1:8">
-      <c r="A12" s="8" t="s">
+      <c r="A12" s="14" t="s">
         <v>46</v>
       </c>
-      <c r="B12" s="9" t="s">
+      <c r="B12" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="C12" s="9" t="s">
+      <c r="C12" s="2" t="s">
         <v>28</v>
       </c>
-      <c r="D12" s="9" t="s">
+      <c r="D12" s="2" t="s">
         <v>47</v>
       </c>
-      <c r="E12" s="9" t="s">
+      <c r="E12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="F12" s="9" t="s">
+      <c r="F12" s="2" t="s">
         <v>45</v>
       </c>
-      <c r="G12" s="10" t="b">
+      <c r="G12" s="2" t="b">
         <v>1</v>
       </c>
-      <c r="H12" s="10"/>
+      <c r="H12" s="8"/>
     </row>
     <row r="13" spans="1:8">
-      <c r="A13" s="8" t="s">
+      <c r="A13" s="16"/>
+      <c r="B13" s="5" t="s">
+        <v>63</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>64</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>65</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" s="5">
+        <v>0</v>
+      </c>
+      <c r="H13" s="18"/>
+    </row>
+    <row r="14" spans="1:8">
+      <c r="A14" s="9" t="s">
         <v>58</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="B14" s="5" t="s">
         <v>57</v>
       </c>
-      <c r="C13" s="9" t="s">
+      <c r="C14" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="9" t="s">
+      <c r="D14" s="5" t="s">
         <v>60</v>
       </c>
-      <c r="E13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="F13" s="9" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="10" t="s">
+      <c r="E14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="F14" s="5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>61</v>
       </c>
-      <c r="H13" s="10" t="s">
+      <c r="H14" s="6" t="s">
         <v>59</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
+  <mergeCells count="3">
     <mergeCell ref="A2:A5"/>
     <mergeCell ref="A6:A11"/>
+    <mergeCell ref="A12:A13"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new IC: BackpackWeapon(v1) new parameter for armor: forcepenlvl new parameter for armor: clamppen
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -1,19 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F5C049FD-EDA1-4BC9-9F51-E14FA9F3ED0B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43242C5-661F-45E9-B281-2CF6F391B941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
-    <sheet name="SwitchableRangedWeapon" sheetId="1" r:id="rId1"/>
+    <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
+    <sheet name="BackpackFedWeapon" sheetId="3" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="90" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="56">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -35,14 +36,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>B</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>modeswitchkey</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>switchableFiremodes</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -51,10 +44,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>firemodeswitchkey</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>burstReload</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -67,10 +56,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>F</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>/</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -115,10 +100,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>A string</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>A list consists of strings</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -151,14 +132,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>The key to cycle between projectiles</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>The key to cycle between firemodes</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>Time required between shots when using Burst firemode</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -179,10 +152,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>To set a key to cycle projectile</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>To list all selectable friemodes</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -199,10 +168,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>All items in Microsoft.Xna.Framework.Input.Keys</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>checkMagCondition</t>
   </si>
   <si>
@@ -269,10 +234,6 @@
   </si>
   <si>
     <t>Lerp(reload, reload*4, 1-reload)</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Deprecated</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
@@ -292,7 +253,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -307,26 +268,13 @@
       <charset val="134"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <sz val="11"/>
-      <name val="等线"/>
-      <family val="3"/>
-      <charset val="134"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="3">
+  <fills count="2">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor theme="1"/>
-        <bgColor indexed="64"/>
-      </patternFill>
     </fill>
   </fills>
   <borders count="12">
@@ -462,7 +410,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -491,16 +439,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
@@ -512,11 +451,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -797,9 +733,9 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H14"/>
-  <sheetFormatPr defaultRowHeight="14"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9EA240FE-1117-4C1F-984C-6020AD1A5D75}">
+  <dimension ref="A1:H20"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5" style="1" bestFit="1" customWidth="1"/>
@@ -812,343 +748,641 @@
     <col min="9" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="E1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="7" t="s">
         <v>16</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="G1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>18</v>
-      </c>
-      <c r="E1" s="8" t="s">
-        <v>19</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>20</v>
-      </c>
-      <c r="G1" s="7" t="s">
-        <v>21</v>
-      </c>
       <c r="H1" s="8" t="s">
-        <v>53</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8">
-      <c r="A2" s="14" t="s">
-        <v>13</v>
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
         <v>0</v>
       </c>
       <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
         <v>24</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="E2" s="2" t="s">
         <v>29</v>
       </c>
-      <c r="E2" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="F2" s="2" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G2" s="3" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>52</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="15"/>
+        <v>43</v>
+      </c>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="12"/>
       <c r="B3" s="1" t="s">
-        <v>48</v>
+        <v>39</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>49</v>
+        <v>40</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>50</v>
+        <v>41</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>51</v>
+        <v>42</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G3" s="4" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="15"/>
+        <v>45</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="13"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>42</v>
+        <v>34</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>37</v>
+        <v>30</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>11</v>
+        <v>7</v>
       </c>
       <c r="G4" s="4">
         <v>0</v>
       </c>
       <c r="H4" s="4"/>
     </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="16"/>
-      <c r="B5" s="10" t="s">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B5" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G5" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H5" s="3"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="12"/>
+      <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="C5" s="10" t="s">
+      <c r="C6" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H6" s="4"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="12"/>
+      <c r="B7" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>22</v>
       </c>
-      <c r="D5" s="10" t="s">
-        <v>31</v>
-      </c>
-      <c r="E5" s="10" t="s">
+      <c r="D7" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="12"/>
+      <c r="B8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="4">
+        <v>0</v>
+      </c>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="13"/>
+      <c r="B9" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="4"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>38</v>
       </c>
-      <c r="F5" s="10" t="s">
-        <v>43</v>
-      </c>
-      <c r="G5" s="11" t="s">
-        <v>10</v>
-      </c>
-      <c r="H5" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>30</v>
-      </c>
-      <c r="E6" s="2" t="s">
-        <v>39</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="G6" s="3" t="s">
-        <v>56</v>
-      </c>
-      <c r="H6" s="3"/>
-    </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="15"/>
-      <c r="B7" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G7" s="4" t="s">
-        <v>11</v>
-      </c>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="15"/>
-      <c r="B8" s="12" t="s">
-        <v>6</v>
-      </c>
-      <c r="C8" s="12" t="s">
+      <c r="E10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F10" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G10" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="8"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="13"/>
+      <c r="B11" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D8" s="12" t="s">
-        <v>32</v>
-      </c>
-      <c r="E8" s="12" t="s">
-        <v>11</v>
-      </c>
-      <c r="F8" s="12" t="s">
-        <v>43</v>
-      </c>
-      <c r="G8" s="13" t="s">
-        <v>2</v>
-      </c>
-      <c r="H8" s="4" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="15"/>
-      <c r="B9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F9" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G9" s="4">
+      <c r="D11" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="5">
         <v>0</v>
       </c>
-      <c r="H9" s="4" t="s">
-        <v>55</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="15"/>
-      <c r="B10" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="F10" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="G10" s="4">
-        <v>0</v>
-      </c>
-      <c r="H10" s="4"/>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="15"/>
-      <c r="B11" s="17" t="s">
-        <v>8</v>
-      </c>
-      <c r="C11" s="17" t="s">
-        <v>28</v>
-      </c>
-      <c r="D11" s="17" t="s">
-        <v>35</v>
-      </c>
-      <c r="E11" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="F11" s="17" t="s">
-        <v>11</v>
-      </c>
-      <c r="G11" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" s="4"/>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="14" t="s">
-        <v>46</v>
-      </c>
-      <c r="B12" s="2" t="s">
-        <v>44</v>
-      </c>
-      <c r="C12" s="2" t="s">
-        <v>28</v>
-      </c>
-      <c r="D12" s="2" t="s">
-        <v>47</v>
-      </c>
-      <c r="E12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="F12" s="2" t="s">
-        <v>45</v>
-      </c>
-      <c r="G12" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" s="8"/>
-    </row>
-    <row r="13" spans="1:8">
-      <c r="A13" s="16"/>
-      <c r="B13" s="5" t="s">
-        <v>63</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>64</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>65</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G13" s="5">
-        <v>0</v>
-      </c>
-      <c r="H13" s="18"/>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="9" t="s">
-        <v>58</v>
-      </c>
-      <c r="B14" s="5" t="s">
-        <v>57</v>
-      </c>
-      <c r="C14" s="5" t="s">
-        <v>27</v>
-      </c>
-      <c r="D14" s="5" t="s">
-        <v>60</v>
-      </c>
-      <c r="E14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="F14" s="5" t="s">
-        <v>11</v>
-      </c>
-      <c r="G14" s="6" t="s">
-        <v>61</v>
-      </c>
-      <c r="H14" s="6" t="s">
-        <v>59</v>
-      </c>
+      <c r="H11" s="10"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H12" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="14"/>
+      <c r="B20" s="14"/>
+      <c r="C20" s="14"/>
+      <c r="D20" s="14"/>
+      <c r="E20" s="14"/>
+      <c r="F20" s="14"/>
+      <c r="G20" s="14"/>
+      <c r="H20" s="14"/>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A6:A11"/>
-    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A2:A4"/>
+    <mergeCell ref="A5:A9"/>
+    <mergeCell ref="A10:A11"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B7A7D7-7F99-4D47-A4D1-1272F654379A}">
+  <dimension ref="A1:H19"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="34.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="44.58203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="27.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="49.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="9" max="16384" width="8.6640625" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="8" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="8" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="8" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="11" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" s="2" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>19</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>29</v>
+      </c>
+      <c r="F2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>7</v>
+      </c>
+      <c r="H2" s="3"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="13"/>
+      <c r="B3" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="4">
+        <v>0</v>
+      </c>
+      <c r="H3" s="4"/>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="11" t="s">
+        <v>11</v>
+      </c>
+      <c r="B4" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>31</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="H4" s="3"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="12"/>
+      <c r="B5" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="F5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="4" t="s">
+        <v>7</v>
+      </c>
+      <c r="H5" s="4"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="12"/>
+      <c r="B6" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="4">
+        <v>0</v>
+      </c>
+      <c r="H6" s="4" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="12"/>
+      <c r="B7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="4">
+        <v>0</v>
+      </c>
+      <c r="H7" s="4"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="13"/>
+      <c r="B8" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="H8" s="4"/>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="11" t="s">
+        <v>37</v>
+      </c>
+      <c r="B9" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D9" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F9" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="G9" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" s="8"/>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="13"/>
+      <c r="B10" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C10" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E10" s="5" t="s">
+        <v>55</v>
+      </c>
+      <c r="F10" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="5">
+        <v>0</v>
+      </c>
+      <c r="H10" s="10"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>51</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="6" t="s">
+        <v>52</v>
+      </c>
+      <c r="H11" s="6" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="14"/>
+      <c r="B17" s="14"/>
+      <c r="C17" s="14"/>
+      <c r="D17" s="14"/>
+      <c r="E17" s="14"/>
+      <c r="F17" s="14"/>
+      <c r="G17" s="14"/>
+      <c r="H17" s="14"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="14"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14"/>
+      <c r="D18" s="14"/>
+      <c r="E18" s="14"/>
+      <c r="F18" s="14"/>
+      <c r="G18" s="14"/>
+      <c r="H18" s="14"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="14"/>
+      <c r="B19" s="14"/>
+      <c r="C19" s="14"/>
+      <c r="D19" s="14"/>
+      <c r="E19" s="14"/>
+      <c r="F19" s="14"/>
+      <c r="G19" s="14"/>
+      <c r="H19" s="14"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="A4:A8"/>
+    <mergeCell ref="A2:A3"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
new IC: ActiveProtectionSystem Compiled all sources
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C43242C5-661F-45E9-B281-2CF6F391B941}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45456301-EF09-45A2-AAD6-4E43226BF7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
     <sheet name="BackpackFedWeapon" sheetId="3" r:id="rId2"/>
+    <sheet name="Sheet1" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="144" uniqueCount="56">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="90">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -246,6 +247,135 @@
   </si>
   <si>
     <t>To modify projectile spread</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Range</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Probility</t>
+  </si>
+  <si>
+    <t>MaxSpeed</t>
+  </si>
+  <si>
+    <t>MinSpeed</t>
+  </si>
+  <si>
+    <t>MinMass</t>
+  </si>
+  <si>
+    <t>MaxMass</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MinSize</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>MaxSize</t>
+  </si>
+  <si>
+    <t>UseOnIntercept</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>RemoveOnIntercept</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>FunctionInInventory</t>
+  </si>
+  <si>
+    <t>float</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Vector2</t>
+  </si>
+  <si>
+    <t>Vector2</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>bool</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define function range of the device</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the success probability of the interception</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the max speed of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the min speed of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the max mass of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the min mass of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the max size of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define the min size of the target</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define whether should perform "Use" on target when interception is successful</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define whether should remove the target when interception is successful</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define whether this device should function when inside an inventory</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>SideNote:</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Also support most parameters in RangedWeapon</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Also support most parameters in Powered</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Max 1, Min 0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Use "meter"(divided by 100) in both X and Y</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>0,0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>1000,1000</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>General</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -277,7 +407,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="12">
+  <borders count="13">
     <border>
       <left/>
       <right/>
@@ -406,11 +536,22 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="29">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -442,18 +583,42 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -775,7 +940,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -801,7 +966,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="12"/>
+      <c r="A3" s="14"/>
       <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
@@ -838,7 +1003,7 @@
       <c r="E4" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F4" s="1" t="s">
+      <c r="F4" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G4" s="4">
@@ -847,7 +1012,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="11" t="s">
+      <c r="A5" s="12" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -871,7 +1036,7 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -893,7 +1058,7 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
+      <c r="A7" s="14"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -917,7 +1082,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="12"/>
+      <c r="A8" s="14"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -961,7 +1126,7 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="11" t="s">
+      <c r="A10" s="12" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1032,41 +1197,67 @@
         <v>50</v>
       </c>
     </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
+    </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14"/>
-      <c r="D20" s="14"/>
-      <c r="E20" s="14"/>
-      <c r="F20" s="14"/>
-      <c r="G20" s="14"/>
-      <c r="H20" s="14"/>
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A2:A4"/>
     <mergeCell ref="A5:A9"/>
     <mergeCell ref="A10:A11"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A16:H16"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1117,7 +1308,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
+      <c r="A2" s="12" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1154,7 +1345,7 @@
       <c r="E3" s="1" t="s">
         <v>30</v>
       </c>
-      <c r="F3" s="1" t="s">
+      <c r="F3" s="5" t="s">
         <v>7</v>
       </c>
       <c r="G3" s="4">
@@ -1163,7 +1354,7 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
+      <c r="A4" s="12" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1187,7 +1378,7 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="12"/>
+      <c r="A5" s="14"/>
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1209,7 +1400,7 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="12"/>
+      <c r="A6" s="14"/>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1233,7 +1424,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="12"/>
+      <c r="A7" s="14"/>
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1277,7 +1468,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="11" t="s">
+      <c r="A9" s="12" t="s">
         <v>37</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1348,44 +1539,359 @@
         <v>50</v>
       </c>
     </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="14"/>
-      <c r="B17" s="14"/>
-      <c r="C17" s="14"/>
-      <c r="D17" s="14"/>
-      <c r="E17" s="14"/>
-      <c r="F17" s="14"/>
-      <c r="G17" s="14"/>
-      <c r="H17" s="14"/>
+      <c r="A17" s="16" t="s">
+        <v>83</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+      <c r="D17" s="11"/>
+      <c r="E17" s="11"/>
+      <c r="F17" s="11"/>
+      <c r="G17" s="11"/>
+      <c r="H17" s="11"/>
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="14"/>
-      <c r="B18" s="14"/>
-      <c r="C18" s="14"/>
-      <c r="D18" s="14"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14"/>
-      <c r="G18" s="14"/>
-      <c r="H18" s="14"/>
+      <c r="A18" s="11"/>
+      <c r="B18" s="11"/>
+      <c r="C18" s="11"/>
+      <c r="D18" s="11"/>
+      <c r="E18" s="11"/>
+      <c r="F18" s="11"/>
+      <c r="G18" s="11"/>
+      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="14"/>
-      <c r="B19" s="14"/>
-      <c r="C19" s="14"/>
-      <c r="D19" s="14"/>
-      <c r="E19" s="14"/>
-      <c r="F19" s="14"/>
-      <c r="G19" s="14"/>
-      <c r="H19" s="14"/>
+      <c r="A19" s="11"/>
+      <c r="B19" s="11"/>
+      <c r="C19" s="11"/>
+      <c r="D19" s="11"/>
+      <c r="E19" s="11"/>
+      <c r="F19" s="11"/>
+      <c r="G19" s="11"/>
+      <c r="H19" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
+  <mergeCells count="5">
     <mergeCell ref="A9:A10"/>
     <mergeCell ref="A4:A8"/>
     <mergeCell ref="A2:A3"/>
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:C17"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4362ADCD-C038-470C-A71D-D8AA3B59ADED}">
+  <dimension ref="A1:H17"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="17.4140625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.25" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="66.4140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="4.9140625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="9.58203125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="37.9140625" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A1" s="7" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="7" t="s">
+        <v>12</v>
+      </c>
+      <c r="C1" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="D1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="E1" s="7" t="s">
+        <v>15</v>
+      </c>
+      <c r="F1" s="7" t="s">
+        <v>16</v>
+      </c>
+      <c r="G1" s="7" t="s">
+        <v>17</v>
+      </c>
+      <c r="H1" s="7" t="s">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A2" s="17" t="s">
+        <v>89</v>
+      </c>
+      <c r="B2" s="18" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="19" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="19" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="2">
+        <v>100</v>
+      </c>
+      <c r="H2" s="26"/>
+    </row>
+    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A3" s="17"/>
+      <c r="B3" s="20" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="21" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" s="21"/>
+      <c r="F3" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="22">
+        <v>1</v>
+      </c>
+      <c r="H3" s="27" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A4" s="17"/>
+      <c r="B4" s="20" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="21" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="22">
+        <v>50</v>
+      </c>
+      <c r="H4" s="27"/>
+    </row>
+    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A5" s="17"/>
+      <c r="B5" s="20" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="21" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="21"/>
+      <c r="F5" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G5" s="22">
+        <v>10</v>
+      </c>
+      <c r="H5" s="27"/>
+    </row>
+    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A6" s="17"/>
+      <c r="B6" s="20" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="21" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="21"/>
+      <c r="F6" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G6" s="22">
+        <v>0</v>
+      </c>
+      <c r="H6" s="27"/>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A7" s="17"/>
+      <c r="B7" s="20" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="21" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="21" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="21"/>
+      <c r="F7" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="22">
+        <v>10000</v>
+      </c>
+      <c r="H7" s="27"/>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A8" s="17"/>
+      <c r="B8" s="20" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="21" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="21" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="21"/>
+      <c r="F8" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="23" t="s">
+        <v>87</v>
+      </c>
+      <c r="H8" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A9" s="17"/>
+      <c r="B9" s="20" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="21" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" s="21" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" s="21"/>
+      <c r="F9" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="23" t="s">
+        <v>88</v>
+      </c>
+      <c r="H9" s="27" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A10" s="17"/>
+      <c r="B10" s="20" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="21" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="21"/>
+      <c r="F10" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="22" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" s="27"/>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A11" s="17"/>
+      <c r="B11" s="20" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="21" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="G11" s="22" t="b">
+        <v>0</v>
+      </c>
+      <c r="H11" s="27"/>
+    </row>
+    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A12" s="17"/>
+      <c r="B12" s="24" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="25" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="25" t="s">
+        <v>81</v>
+      </c>
+      <c r="E12" s="25"/>
+      <c r="F12" s="25" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="5" t="b">
+        <v>0</v>
+      </c>
+      <c r="H12" s="28"/>
+    </row>
+    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A16" s="15" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15"/>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="15" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="15"/>
+      <c r="C17" s="15"/>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="A16:H16"/>
+    <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A2:A12"/>
+  </mergeCells>
+  <phoneticPr fontId="1" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Fixed potential mem leaks in APS Fixed mistakes in Armors Implemented CreateExplosionOnIntercept Implemented InterceptOnlyApproaching
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45456301-EF09-45A2-AAD6-4E43226BF7CF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38325CE-EAC6-4CE6-8430-69A400C01451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
     <sheet name="BackpackFedWeapon" sheetId="3" r:id="rId2"/>
-    <sheet name="Sheet1" sheetId="5" r:id="rId3"/>
+    <sheet name="APS" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="208" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -367,15 +367,31 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>0,0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>1000,1000</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>General</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Also support Explosion as a subelement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>InterceptOnlyApproaching</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CreateExplosionsOnIntercept</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The device will only intercept projectiles/throwables flying towards it if true</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>An explosion will be create at the position where the target was intercepted</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Should always define an Explosion as an subelement</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -551,7 +567,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -586,39 +602,49 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="常规" xfId="0" builtinId="0"/>
@@ -940,7 +966,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="17" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -966,7 +992,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="14"/>
+      <c r="A3" s="18"/>
       <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
@@ -990,7 +1016,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="13"/>
+      <c r="A4" s="19"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1012,7 +1038,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="12" t="s">
+      <c r="A5" s="17" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1036,7 +1062,7 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1058,7 +1084,7 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1082,7 +1108,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="14"/>
+      <c r="A8" s="18"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1104,7 +1130,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="13"/>
+      <c r="A9" s="19"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1126,7 +1152,7 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="12" t="s">
+      <c r="A10" s="17" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1150,7 +1176,7 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="13"/>
+      <c r="A11" s="19"/>
       <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
@@ -1198,23 +1224,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1308,7 +1334,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="12" t="s">
+      <c r="A2" s="17" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1332,7 +1358,7 @@
       <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="13"/>
+      <c r="A3" s="19"/>
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1354,7 +1380,7 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="12" t="s">
+      <c r="A4" s="17" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1378,7 +1404,7 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="14"/>
+      <c r="A5" s="18"/>
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1400,7 +1426,7 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="14"/>
+      <c r="A6" s="18"/>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1424,7 +1450,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="14"/>
+      <c r="A7" s="18"/>
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1446,7 +1472,7 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="13"/>
+      <c r="A8" s="19"/>
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
@@ -1468,7 +1494,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="12" t="s">
+      <c r="A9" s="17" t="s">
         <v>37</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1492,7 +1518,7 @@
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="13"/>
+      <c r="A10" s="19"/>
       <c r="B10" s="5" t="s">
         <v>53</v>
       </c>
@@ -1540,23 +1566,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
+      <c r="A16" s="16" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="16" t="s">
+      <c r="A17" s="20" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="16"/>
-      <c r="C17" s="16"/>
+      <c r="B17" s="20"/>
+      <c r="C17" s="20"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1599,297 +1625,329 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4362ADCD-C038-470C-A71D-D8AA3B59ADED}">
-  <dimension ref="A1:H17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="17.4140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.9140625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="12.25" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="66.4140625" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="4.9140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="15.5" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="9.58203125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="37.9140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="15.5" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.58203125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="44.75" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" s="8" t="s">
         <v>10</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="8" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="7" t="s">
+      <c r="C1" s="8" t="s">
         <v>13</v>
       </c>
-      <c r="D1" s="7" t="s">
+      <c r="D1" s="8" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="7" t="s">
-        <v>15</v>
-      </c>
-      <c r="F1" s="7" t="s">
+      <c r="E1" s="8" t="s">
         <v>16</v>
       </c>
-      <c r="G1" s="7" t="s">
+      <c r="F1" s="8" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="7" t="s">
+      <c r="G1" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="17" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B2" s="12" t="s">
+        <v>56</v>
+      </c>
+      <c r="C2" s="13" t="s">
+        <v>67</v>
+      </c>
+      <c r="D2" s="13" t="s">
+        <v>71</v>
+      </c>
+      <c r="E2" s="13" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="3">
+        <v>100</v>
+      </c>
+      <c r="G2" s="24"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="31"/>
+      <c r="B3" s="14" t="s">
+        <v>57</v>
+      </c>
+      <c r="C3" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D3" s="23" t="s">
+        <v>72</v>
+      </c>
+      <c r="E3" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="4">
+        <v>1</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="31"/>
+      <c r="B4" s="14" t="s">
+        <v>58</v>
+      </c>
+      <c r="C4" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D4" s="23" t="s">
+        <v>73</v>
+      </c>
+      <c r="E4" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="4">
+        <v>50</v>
+      </c>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="31"/>
+      <c r="B5" s="14" t="s">
+        <v>59</v>
+      </c>
+      <c r="C5" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D5" s="23" t="s">
+        <v>74</v>
+      </c>
+      <c r="E5" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="4">
+        <v>10</v>
+      </c>
+      <c r="G5" s="25"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="31"/>
+      <c r="B6" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C6" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D6" s="23" t="s">
+        <v>75</v>
+      </c>
+      <c r="E6" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="4">
+        <v>0</v>
+      </c>
+      <c r="G6" s="25"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="31"/>
+      <c r="B7" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C7" s="23" t="s">
+        <v>67</v>
+      </c>
+      <c r="D7" s="23" t="s">
+        <v>76</v>
+      </c>
+      <c r="E7" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="4">
+        <v>10000</v>
+      </c>
+      <c r="G7" s="25"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="31"/>
+      <c r="B8" s="14" t="s">
+        <v>63</v>
+      </c>
+      <c r="C8" s="23" t="s">
+        <v>68</v>
+      </c>
+      <c r="D8" s="23" t="s">
+        <v>77</v>
+      </c>
+      <c r="E8" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="25" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="31"/>
+      <c r="B9" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" s="23" t="s">
+        <v>69</v>
+      </c>
+      <c r="D9" s="23" t="s">
+        <v>78</v>
+      </c>
+      <c r="E9" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="27" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="25" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="31"/>
+      <c r="B10" s="14" t="s">
+        <v>64</v>
+      </c>
+      <c r="C10" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D10" s="23" t="s">
+        <v>79</v>
+      </c>
+      <c r="E10" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="4" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="31"/>
+      <c r="B11" s="14" t="s">
+        <v>65</v>
+      </c>
+      <c r="C11" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D11" s="23" t="s">
+        <v>80</v>
+      </c>
+      <c r="E11" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G11" s="25"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="31"/>
+      <c r="B12" s="14" t="s">
+        <v>66</v>
+      </c>
+      <c r="C12" s="23" t="s">
+        <v>70</v>
+      </c>
+      <c r="D12" s="23" t="s">
+        <v>81</v>
+      </c>
+      <c r="E12" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G12" s="25"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="31"/>
+      <c r="B13" s="14" t="s">
         <v>89</v>
       </c>
-      <c r="B2" s="18" t="s">
-        <v>56</v>
-      </c>
-      <c r="C2" s="19" t="s">
-        <v>67</v>
-      </c>
-      <c r="D2" s="19" t="s">
-        <v>71</v>
-      </c>
-      <c r="E2" s="19"/>
-      <c r="F2" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="2">
-        <v>100</v>
-      </c>
-      <c r="H2" s="26"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="17"/>
-      <c r="B3" s="20" t="s">
-        <v>57</v>
-      </c>
-      <c r="C3" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D3" s="21" t="s">
-        <v>72</v>
-      </c>
-      <c r="E3" s="21"/>
-      <c r="F3" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="22">
+      <c r="C13" s="21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D13" s="21" t="s">
+        <v>91</v>
+      </c>
+      <c r="E13" s="21" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="28" t="b">
         <v>1</v>
       </c>
-      <c r="H3" s="27" t="s">
-        <v>85</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="17"/>
-      <c r="B4" s="20" t="s">
-        <v>58</v>
-      </c>
-      <c r="C4" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D4" s="21" t="s">
-        <v>73</v>
-      </c>
-      <c r="E4" s="21"/>
-      <c r="F4" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G4" s="22">
-        <v>50</v>
-      </c>
-      <c r="H4" s="27"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="17"/>
-      <c r="B5" s="20" t="s">
-        <v>59</v>
-      </c>
-      <c r="C5" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D5" s="21" t="s">
-        <v>74</v>
-      </c>
-      <c r="E5" s="21"/>
-      <c r="F5" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="22">
-        <v>10</v>
-      </c>
-      <c r="H5" s="27"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="17"/>
-      <c r="B6" s="20" t="s">
-        <v>61</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>75</v>
-      </c>
-      <c r="E6" s="21"/>
-      <c r="F6" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="22">
+      <c r="G13" s="25"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="32"/>
+      <c r="B14" s="15" t="s">
+        <v>90</v>
+      </c>
+      <c r="C14" s="26" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" s="26" t="s">
+        <v>92</v>
+      </c>
+      <c r="E14" s="26" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="29" t="b">
         <v>0</v>
       </c>
-      <c r="H6" s="27"/>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="17"/>
-      <c r="B7" s="20" t="s">
-        <v>60</v>
-      </c>
-      <c r="C7" s="21" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" s="21" t="s">
-        <v>76</v>
-      </c>
-      <c r="E7" s="21"/>
-      <c r="F7" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="22">
-        <v>10000</v>
-      </c>
-      <c r="H7" s="27"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="17"/>
-      <c r="B8" s="20" t="s">
-        <v>63</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>68</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>77</v>
-      </c>
-      <c r="E8" s="21"/>
-      <c r="F8" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="23" t="s">
-        <v>87</v>
-      </c>
-      <c r="H8" s="27" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="17"/>
-      <c r="B9" s="20" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" s="21" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" s="21" t="s">
-        <v>78</v>
-      </c>
-      <c r="E9" s="21"/>
-      <c r="F9" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="23" t="s">
+      <c r="G14" s="22" t="s">
+        <v>93</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16" s="16" t="s">
+        <v>82</v>
+      </c>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16"/>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A17" s="16" t="s">
+        <v>84</v>
+      </c>
+      <c r="B17" s="16"/>
+      <c r="C17" s="16"/>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
+      <c r="A18" s="16" t="s">
         <v>88</v>
       </c>
-      <c r="H9" s="27" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="17"/>
-      <c r="B10" s="20" t="s">
-        <v>64</v>
-      </c>
-      <c r="C10" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" s="21" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" s="21"/>
-      <c r="F10" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" s="27"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="17"/>
-      <c r="B11" s="20" t="s">
-        <v>65</v>
-      </c>
-      <c r="C11" s="21" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" s="21" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" s="21"/>
-      <c r="F11" s="21" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="22" t="b">
-        <v>0</v>
-      </c>
-      <c r="H11" s="27"/>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A12" s="17"/>
-      <c r="B12" s="24" t="s">
-        <v>66</v>
-      </c>
-      <c r="C12" s="25" t="s">
-        <v>70</v>
-      </c>
-      <c r="D12" s="25" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" s="25"/>
-      <c r="F12" s="25" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="5" t="b">
-        <v>0</v>
-      </c>
-      <c r="H12" s="28"/>
-    </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="15" t="s">
-        <v>82</v>
-      </c>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15"/>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="15" t="s">
-        <v>84</v>
-      </c>
-      <c r="B17" s="15"/>
-      <c r="C17" s="15"/>
+      <c r="B18" s="16"/>
+      <c r="C18" s="16"/>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A16:H16"/>
+  <mergeCells count="4">
+    <mergeCell ref="A18:C18"/>
+    <mergeCell ref="A16:G16"/>
     <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A2:A12"/>
+    <mergeCell ref="A2:A14"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Fixed sequence issue in APS Added an property to set amount of condition reduced when interception is successful
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,14 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E38325CE-EAC6-4CE6-8430-69A400C01451}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837E951D-C10F-48DB-B19B-58C4FFB24887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
     <sheet name="BackpackFedWeapon" sheetId="3" r:id="rId2"/>
-    <sheet name="APS" sheetId="5" r:id="rId3"/>
+    <sheet name="ActiveProtectionSystem" sheetId="5" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="217" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -392,6 +392,13 @@
   </si>
   <si>
     <t>Should always define an Explosion as an subelement</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>ReduceConditionOnIntercept</t>
+  </si>
+  <si>
+    <t>Define the amount of condition reduced on target when interception is successful</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -567,7 +574,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="32">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -612,6 +619,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
@@ -958,7 +974,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="28" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -984,7 +1000,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="26"/>
+      <c r="A3" s="29"/>
       <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
@@ -1008,7 +1024,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="27"/>
+      <c r="A4" s="30"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1030,7 +1046,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="25" t="s">
+      <c r="A5" s="28" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1054,7 +1070,7 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1076,7 +1092,7 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
+      <c r="A7" s="29"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1100,7 +1116,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="26"/>
+      <c r="A8" s="29"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1122,7 +1138,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="27"/>
+      <c r="A9" s="30"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1144,7 +1160,7 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="25" t="s">
+      <c r="A10" s="28" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1168,7 +1184,7 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="27"/>
+      <c r="A11" s="30"/>
       <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
@@ -1216,23 +1232,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1326,7 +1342,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="28" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1350,7 +1366,7 @@
       <c r="H2" s="3"/>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="27"/>
+      <c r="A3" s="30"/>
       <c r="B3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1372,7 +1388,7 @@
       <c r="H3" s="4"/>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="25" t="s">
+      <c r="A4" s="28" t="s">
         <v>11</v>
       </c>
       <c r="B4" s="2" t="s">
@@ -1396,7 +1412,7 @@
       <c r="H4" s="3"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="26"/>
+      <c r="A5" s="29"/>
       <c r="B5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1418,7 +1434,7 @@
       <c r="H5" s="4"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
+      <c r="A6" s="29"/>
       <c r="B6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1442,7 +1458,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
+      <c r="A7" s="29"/>
       <c r="B7" s="1" t="s">
         <v>6</v>
       </c>
@@ -1464,7 +1480,7 @@
       <c r="H7" s="4"/>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="27"/>
+      <c r="A8" s="30"/>
       <c r="B8" s="1" t="s">
         <v>5</v>
       </c>
@@ -1486,7 +1502,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
+      <c r="A9" s="28" t="s">
         <v>37</v>
       </c>
       <c r="B9" s="2" t="s">
@@ -1510,7 +1526,7 @@
       <c r="H9" s="8"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
+      <c r="A10" s="30"/>
       <c r="B10" s="5" t="s">
         <v>53</v>
       </c>
@@ -1558,23 +1574,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-      <c r="H16" s="21"/>
+      <c r="B16" s="24"/>
+      <c r="C16" s="24"/>
+      <c r="D16" s="24"/>
+      <c r="E16" s="24"/>
+      <c r="F16" s="24"/>
+      <c r="G16" s="24"/>
+      <c r="H16" s="24"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="31" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="28"/>
-      <c r="C17" s="28"/>
+      <c r="B17" s="31"/>
+      <c r="C17" s="31"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1617,7 +1633,7 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{4362ADCD-C038-470C-A71D-D8AA3B59ADED}">
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.1640625" bestFit="1" customWidth="1"/>
@@ -1653,7 +1669,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="22" t="s">
+      <c r="A2" s="25" t="s">
         <v>87</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -1665,7 +1681,7 @@
       <c r="D2" s="13" t="s">
         <v>71</v>
       </c>
-      <c r="E2" s="13" t="s">
+      <c r="E2" s="21" t="s">
         <v>7</v>
       </c>
       <c r="F2" s="3">
@@ -1674,7 +1690,7 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="23"/>
+      <c r="A3" s="26"/>
       <c r="B3" s="14" t="s">
         <v>57</v>
       </c>
@@ -1684,7 +1700,7 @@
       <c r="D3" t="s">
         <v>72</v>
       </c>
-      <c r="E3" t="s">
+      <c r="E3" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F3" s="4">
@@ -1695,7 +1711,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="23"/>
+      <c r="A4" s="26"/>
       <c r="B4" s="14" t="s">
         <v>58</v>
       </c>
@@ -1705,7 +1721,7 @@
       <c r="D4" t="s">
         <v>73</v>
       </c>
-      <c r="E4" t="s">
+      <c r="E4" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F4" s="4">
@@ -1714,7 +1730,7 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="23"/>
+      <c r="A5" s="26"/>
       <c r="B5" s="14" t="s">
         <v>59</v>
       </c>
@@ -1724,7 +1740,7 @@
       <c r="D5" t="s">
         <v>74</v>
       </c>
-      <c r="E5" t="s">
+      <c r="E5" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F5" s="4">
@@ -1733,7 +1749,7 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="23"/>
+      <c r="A6" s="26"/>
       <c r="B6" s="14" t="s">
         <v>61</v>
       </c>
@@ -1743,7 +1759,7 @@
       <c r="D6" t="s">
         <v>75</v>
       </c>
-      <c r="E6" t="s">
+      <c r="E6" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F6" s="4">
@@ -1752,57 +1768,55 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="23"/>
+      <c r="A7" s="26"/>
       <c r="B7" s="14" t="s">
-        <v>60</v>
+        <v>94</v>
       </c>
       <c r="C7" t="s">
         <v>67</v>
       </c>
       <c r="D7" t="s">
+        <v>95</v>
+      </c>
+      <c r="E7" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="4">
+        <v>0</v>
+      </c>
+      <c r="G7" s="18"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="26"/>
+      <c r="B8" s="14" t="s">
+        <v>60</v>
+      </c>
+      <c r="C8" t="s">
+        <v>67</v>
+      </c>
+      <c r="D8" t="s">
         <v>76</v>
       </c>
-      <c r="E7" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="4">
+      <c r="E8" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="4">
         <v>10000</v>
       </c>
-      <c r="G7" s="18"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="23"/>
-      <c r="B8" s="14" t="s">
+      <c r="G8" s="18"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="26"/>
+      <c r="B9" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C8" t="s">
+      <c r="C9" t="s">
         <v>68</v>
       </c>
-      <c r="D8" t="s">
+      <c r="D9" t="s">
         <v>77</v>
       </c>
-      <c r="E8" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="23"/>
-      <c r="B9" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C9" t="s">
-        <v>69</v>
-      </c>
-      <c r="D9" t="s">
-        <v>78</v>
-      </c>
-      <c r="E9" t="s">
+      <c r="E9" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F9" s="20" t="s">
@@ -1813,55 +1827,57 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="23"/>
+      <c r="A10" s="26"/>
       <c r="B10" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C10" t="s">
+        <v>69</v>
+      </c>
+      <c r="D10" t="s">
+        <v>78</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="26"/>
+      <c r="B11" s="14" t="s">
         <v>64</v>
-      </c>
-      <c r="C10" t="s">
-        <v>70</v>
-      </c>
-      <c r="D10" t="s">
-        <v>79</v>
-      </c>
-      <c r="E10" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" s="18"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="23"/>
-      <c r="B11" s="14" t="s">
-        <v>65</v>
       </c>
       <c r="C11" t="s">
         <v>70</v>
       </c>
       <c r="D11" t="s">
-        <v>80</v>
-      </c>
-      <c r="E11" t="s">
+        <v>79</v>
+      </c>
+      <c r="E11" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F11" s="4" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="23"/>
+      <c r="A12" s="26"/>
       <c r="B12" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C12" t="s">
         <v>70</v>
       </c>
       <c r="D12" t="s">
-        <v>81</v>
-      </c>
-      <c r="E12" t="s">
+        <v>80</v>
+      </c>
+      <c r="E12" s="22" t="s">
         <v>7</v>
       </c>
       <c r="F12" s="4" t="b">
@@ -1870,76 +1886,103 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="23"/>
+      <c r="A13" s="26"/>
       <c r="B13" s="14" t="s">
-        <v>89</v>
+        <v>66</v>
       </c>
       <c r="C13" t="s">
         <v>70</v>
       </c>
       <c r="D13" t="s">
+        <v>81</v>
+      </c>
+      <c r="E13" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="4" t="b">
+        <v>0</v>
+      </c>
+      <c r="G13" s="18"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="26"/>
+      <c r="B14" s="14" t="s">
+        <v>89</v>
+      </c>
+      <c r="C14" t="s">
+        <v>70</v>
+      </c>
+      <c r="D14" t="s">
         <v>91</v>
       </c>
-      <c r="E13" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="4" t="b">
+      <c r="E14" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="4" t="b">
         <v>1</v>
       </c>
-      <c r="G13" s="18"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="24"/>
-      <c r="B14" s="15" t="s">
+      <c r="G14" s="18"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="27"/>
+      <c r="B15" s="15" t="s">
         <v>90</v>
       </c>
-      <c r="C14" s="19" t="s">
+      <c r="C15" s="19" t="s">
         <v>70</v>
       </c>
-      <c r="D14" s="19" t="s">
+      <c r="D15" s="19" t="s">
         <v>92</v>
       </c>
-      <c r="E14" s="19" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="6" t="b">
+      <c r="E15" s="23" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="6" t="b">
         <v>0</v>
       </c>
-      <c r="G14" s="16" t="s">
+      <c r="G15" s="16" t="s">
         <v>93</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="21" t="s">
+      <c r="A16" s="1"/>
+      <c r="F16" s="1"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17" s="1"/>
+      <c r="F17" s="1"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="21"/>
-      <c r="C16" s="21"/>
-      <c r="D16" s="21"/>
-      <c r="E16" s="21"/>
-      <c r="F16" s="21"/>
-      <c r="G16" s="21"/>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="21" t="s">
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20" s="24" t="s">
         <v>84</v>
       </c>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="21" t="s">
+      <c r="B20" s="24"/>
+      <c r="C20" s="24"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21" s="24" t="s">
         <v>88</v>
       </c>
-      <c r="B18" s="21"/>
-      <c r="C18" s="21"/>
+      <c r="B21" s="24"/>
+      <c r="C21" s="24"/>
     </row>
   </sheetData>
   <mergeCells count="4">
-    <mergeCell ref="A18:C18"/>
-    <mergeCell ref="A16:G16"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A2:A14"/>
+    <mergeCell ref="A21:C21"/>
+    <mergeCell ref="A19:G19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A2:A15"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
updated doc backpack will be considered to have only 1 slot if UseAllBackpackAvailable is True
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{837E951D-C10F-48DB-B19B-58C4FFB24887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EFAE56-797D-451C-8938-AAD17A743BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="221" uniqueCount="96">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="107">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -399,6 +399,50 @@
   </si>
   <si>
     <t>Define the amount of condition reduced on target when interception is successful</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>requiredBackPackID</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Identifiers of backpacks the weapon will attempt to draw ammo from</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>allowedSelfContainerIndex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Index of weapon's own container slots the weapon can select from</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>CurrentSlotIndex</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>UseAllBackpackAvailable</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Define whether the weapon will consider every projectile in the backpack valid</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Index of slot the weapon is currently using</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>If true, backpack will be considered having only 1 slot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Upper cap will dynamically change with different backpack</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>If the backpack you are wearing is not in this list, the backpack will be considered having 0 slot</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -574,7 +618,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="32">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -632,6 +676,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -652,6 +702,9 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -974,7 +1027,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+      <c r="A2" s="30" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1000,7 +1053,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="29"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1" t="s">
         <v>39</v>
       </c>
@@ -1024,7 +1077,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="30"/>
+      <c r="A4" s="32"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1046,7 +1099,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="28" t="s">
+      <c r="A5" s="30" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1070,7 +1123,7 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1092,7 +1145,7 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1116,7 +1169,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="29"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1138,7 +1191,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="30"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1160,7 +1213,7 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="28" t="s">
+      <c r="A10" s="30" t="s">
         <v>37</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1184,7 +1237,7 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="30"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5" t="s">
         <v>53</v>
       </c>
@@ -1232,23 +1285,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+      <c r="A16" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="31" t="s">
+      <c r="A17" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1301,311 +1354,310 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B7A7D7-7F99-4D47-A4D1-1272F654379A}">
-  <dimension ref="A1:H19"/>
+  <dimension ref="A1:H23"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="21.5" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="34.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="20.08203125" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="31.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="44.58203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="27.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="19.4140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="27.25" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="79.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="49.25" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="8.6640625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A1" s="7" t="s">
         <v>10</v>
       </c>
       <c r="B1" s="7" t="s">
         <v>12</v>
       </c>
-      <c r="C1" s="8" t="s">
+      <c r="C1" s="7" t="s">
         <v>13</v>
       </c>
       <c r="D1" s="7" t="s">
         <v>14</v>
       </c>
-      <c r="E1" s="8" t="s">
-        <v>15</v>
+      <c r="E1" s="7" t="s">
+        <v>16</v>
       </c>
       <c r="F1" s="7" t="s">
-        <v>16</v>
-      </c>
-      <c r="G1" s="7" t="s">
         <v>17</v>
       </c>
-      <c r="H1" s="8" t="s">
+      <c r="G1" s="8" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="28" t="s">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2" s="30" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="34" t="s">
+        <v>96</v>
+      </c>
+      <c r="C2" s="34" t="s">
+        <v>18</v>
+      </c>
+      <c r="D2" s="34" t="s">
+        <v>97</v>
+      </c>
+      <c r="E2" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>106</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="31"/>
+      <c r="B3" s="34" t="s">
+        <v>98</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>40</v>
+      </c>
+      <c r="D3" s="34" t="s">
+        <v>99</v>
+      </c>
+      <c r="E3" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="25"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="31"/>
+      <c r="B4" s="34" t="s">
+        <v>100</v>
+      </c>
+      <c r="C4" s="34" t="s">
+        <v>21</v>
+      </c>
+      <c r="D4" s="34" t="s">
+        <v>103</v>
+      </c>
+      <c r="E4" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="34">
         <v>0</v>
       </c>
-      <c r="C2" s="2" t="s">
-        <v>19</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>24</v>
-      </c>
-      <c r="E2" s="2" t="s">
-        <v>29</v>
-      </c>
-      <c r="F2" s="2" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="3" t="s">
-        <v>7</v>
-      </c>
-      <c r="H2" s="3"/>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="30"/>
-      <c r="B3" s="1" t="s">
+      <c r="G4" s="25" t="s">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="32"/>
+      <c r="B5" s="5" t="s">
+        <v>101</v>
+      </c>
+      <c r="C5" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D5" s="5" t="s">
+        <v>102</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="5" t="b">
         <v>1</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="G5" s="10" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="30" t="s">
+        <v>11</v>
+      </c>
+      <c r="B6" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="2" t="s">
+        <v>47</v>
+      </c>
+      <c r="G6" s="8"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="31"/>
+      <c r="B7" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D3" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E3" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="F3" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="4">
+      <c r="D7" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F7" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="G7" s="25"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="31"/>
+      <c r="B8" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="34">
         <v>0</v>
       </c>
-      <c r="H3" s="4"/>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="28" t="s">
-        <v>11</v>
-      </c>
-      <c r="B4" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C4" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E4" s="2" t="s">
-        <v>31</v>
-      </c>
-      <c r="F4" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>47</v>
-      </c>
-      <c r="H4" s="3"/>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="29"/>
-      <c r="B5" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C5" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="D5" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E5" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="F5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G5" s="4" t="s">
-        <v>7</v>
-      </c>
-      <c r="H5" s="4"/>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="29"/>
-      <c r="B6" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C6" s="1" t="s">
+      <c r="G8" s="25" t="s">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="31"/>
+      <c r="B9" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="34">
+        <v>0</v>
+      </c>
+      <c r="G9" s="25"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="31"/>
+      <c r="B10" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>28</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="34" t="b">
+        <v>1</v>
+      </c>
+      <c r="G10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="30" t="s">
+        <v>37</v>
+      </c>
+      <c r="B11" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F11" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G11" s="8"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="32"/>
+      <c r="B12" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="C12" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D6" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F6" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G6" s="4">
+      <c r="D12" s="5" t="s">
+        <v>54</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="5">
         <v>0</v>
       </c>
-      <c r="H6" s="4" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="29"/>
-      <c r="B7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C7" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D7" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="4">
-        <v>0</v>
-      </c>
-      <c r="H7" s="4"/>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="30"/>
-      <c r="B8" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="G8" s="4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" s="4"/>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="28" t="s">
-        <v>37</v>
-      </c>
-      <c r="B9" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C9" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D9" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F9" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="G9" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" s="8"/>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="30"/>
-      <c r="B10" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C10" s="5" t="s">
+      <c r="G12" s="10"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="9" t="s">
+        <v>49</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>48</v>
+      </c>
+      <c r="C13" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="D10" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E10" s="5" t="s">
-        <v>55</v>
-      </c>
-      <c r="F10" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="5">
-        <v>0</v>
-      </c>
-      <c r="H10" s="10"/>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="9" t="s">
-        <v>49</v>
-      </c>
-      <c r="B11" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="D13" s="5" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F11" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G11" s="6" t="s">
+      <c r="E13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="6" t="s">
         <v>52</v>
       </c>
-      <c r="H11" s="6" t="s">
+      <c r="G13" s="6" t="s">
         <v>50</v>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="24" t="s">
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="24" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="24"/>
-      <c r="C16" s="24"/>
-      <c r="D16" s="24"/>
-      <c r="E16" s="24"/>
-      <c r="F16" s="24"/>
-      <c r="G16" s="24"/>
-      <c r="H16" s="24"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="31" t="s">
+      <c r="B17" s="24"/>
+      <c r="C17" s="24"/>
+      <c r="D17" s="24"/>
+      <c r="E17" s="24"/>
+      <c r="F17" s="24"/>
+      <c r="G17" s="24"/>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="33" t="s">
         <v>83</v>
       </c>
-      <c r="B17" s="31"/>
-      <c r="C17" s="31"/>
-      <c r="D17" s="11"/>
-      <c r="E17" s="11"/>
-      <c r="F17" s="11"/>
-      <c r="G17" s="11"/>
-      <c r="H17" s="11"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="11"/>
-      <c r="B18" s="11"/>
-      <c r="C18" s="11"/>
+      <c r="B18" s="33"/>
+      <c r="C18" s="33"/>
       <c r="D18" s="11"/>
       <c r="E18" s="11"/>
       <c r="F18" s="11"/>
       <c r="G18" s="11"/>
-      <c r="H18" s="11"/>
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A19" s="11"/>
@@ -1615,15 +1667,32 @@
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
       <c r="G19" s="11"/>
-      <c r="H19" s="11"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="11"/>
+      <c r="B20" s="11"/>
+      <c r="C20" s="11"/>
+      <c r="D20" s="11"/>
+      <c r="E20" s="11"/>
+      <c r="F20" s="11"/>
+      <c r="G20" s="11"/>
+      <c r="H20" s="24"/>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H21" s="11"/>
+    </row>
+    <row r="22" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H22" s="11"/>
+    </row>
+    <row r="23" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H23" s="11"/>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A4:A8"/>
-    <mergeCell ref="A2:A3"/>
-    <mergeCell ref="A16:H16"/>
-    <mergeCell ref="A17:C17"/>
+  <mergeCells count="4">
+    <mergeCell ref="A2:A5"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="A6:A10"/>
+    <mergeCell ref="A18:C18"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1669,7 +1738,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="25" t="s">
+      <c r="A2" s="27" t="s">
         <v>87</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -1690,7 +1759,7 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="26"/>
+      <c r="A3" s="28"/>
       <c r="B3" s="14" t="s">
         <v>57</v>
       </c>
@@ -1711,7 +1780,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="26"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="14" t="s">
         <v>58</v>
       </c>
@@ -1730,7 +1799,7 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="26"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="14" t="s">
         <v>59</v>
       </c>
@@ -1749,7 +1818,7 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="26"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="14" t="s">
         <v>61</v>
       </c>
@@ -1768,7 +1837,7 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="26"/>
+      <c r="A7" s="28"/>
       <c r="B7" s="14" t="s">
         <v>94</v>
       </c>
@@ -1787,7 +1856,7 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="26"/>
+      <c r="A8" s="28"/>
       <c r="B8" s="14" t="s">
         <v>60</v>
       </c>
@@ -1806,7 +1875,7 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="26"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="14" t="s">
         <v>63</v>
       </c>
@@ -1827,7 +1896,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="14" t="s">
         <v>62</v>
       </c>
@@ -1848,7 +1917,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="26"/>
+      <c r="A11" s="28"/>
       <c r="B11" s="14" t="s">
         <v>64</v>
       </c>
@@ -1867,7 +1936,7 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="26"/>
+      <c r="A12" s="28"/>
       <c r="B12" s="14" t="s">
         <v>65</v>
       </c>
@@ -1886,7 +1955,7 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="26"/>
+      <c r="A13" s="28"/>
       <c r="B13" s="14" t="s">
         <v>66</v>
       </c>
@@ -1905,7 +1974,7 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="26"/>
+      <c r="A14" s="28"/>
       <c r="B14" s="14" t="s">
         <v>89</v>
       </c>
@@ -1924,7 +1993,7 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="27"/>
+      <c r="A15" s="29"/>
       <c r="B15" s="15" t="s">
         <v>90</v>
       </c>
@@ -1953,29 +2022,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="24" t="s">
+      <c r="A19" s="26" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
-      <c r="E19" s="24"/>
-      <c r="F19" s="24"/>
-      <c r="G19" s="24"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="24" t="s">
+      <c r="A20" s="26" t="s">
         <v>84</v>
       </c>
-      <c r="B20" s="24"/>
-      <c r="C20" s="24"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="24" t="s">
+      <c r="A21" s="26" t="s">
         <v>88</v>
       </c>
-      <c r="B21" s="24"/>
-      <c r="C21" s="24"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
Removed accidentally added test item BackpackFedWeapon: Allowed backpack will now defined with tag instead of Identifier Renamed requiredBackPackID to allowedBackPackTags Added allowedProjectileTags to define the projectile the weapon can shoot Improved CurrentSlotIndex setter Misc adjustments on logics
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla Components Expanded\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla_Components_Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{32EFAE56-797D-451C-8938-AAD17A743BB8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0C9189-882F-4FFA-A1A9-8B9389ADA110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="222" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="111">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -113,10 +113,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>A integer larger than 0</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>A float</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -402,14 +398,6 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>requiredBackPackID</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
-    <t>Identifiers of backpacks the weapon will attempt to draw ammo from</t>
-    <phoneticPr fontId="1" type="noConversion"/>
-  </si>
-  <si>
     <t>allowedSelfContainerIndex</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
@@ -442,7 +430,35 @@
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
   <si>
-    <t>If the backpack you are wearing is not in this list, the backpack will be considered having 0 slot</t>
+    <t>A list of Tags</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tags of backpacks the weapon is allowed to attempt to draw ammo from</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>allowedBackPackTags</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>allowedProjectileTags</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Tags of ammo the weapon is allowed to shoot</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The weapon will shoot whatever it can find in the backpack if not defined</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>The backpack you wear will be considered having 0 slot if does not have tags in this list/this is not defined</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>An integer larger than 0</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -618,7 +634,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="35">
+  <cellXfs count="37">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -679,6 +695,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -692,19 +720,13 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1023,11 +1045,11 @@
         <v>17</v>
       </c>
       <c r="H1" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="26" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1037,10 +1059,10 @@
         <v>19</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="F2" s="2" t="s">
         <v>7</v>
@@ -1049,23 +1071,23 @@
         <v>7</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="31"/>
+      <c r="A3" s="27"/>
       <c r="B3" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="C3" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="C3" s="1" t="s">
+      <c r="D3" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="D3" s="1" t="s">
+      <c r="E3" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="E3" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="F3" s="1" t="s">
         <v>7</v>
       </c>
@@ -1073,22 +1095,22 @@
         <v>7</v>
       </c>
       <c r="H3" s="4" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F4" s="5" t="s">
         <v>7</v>
@@ -1099,7 +1121,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="30" t="s">
+      <c r="A5" s="26" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1109,32 +1131,32 @@
         <v>18</v>
       </c>
       <c r="D5" s="2" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="E5" s="2" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="F5" s="1" t="s">
         <v>8</v>
       </c>
       <c r="G5" s="3" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="31"/>
+      <c r="A6" s="27"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>21</v>
+        <v>110</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="F6" s="1" t="s">
         <v>7</v>
@@ -1145,15 +1167,15 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="31"/>
+      <c r="A7" s="27"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E7" s="1" t="s">
         <v>7</v>
@@ -1165,19 +1187,19 @@
         <v>0</v>
       </c>
       <c r="H7" s="4" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="31"/>
+      <c r="A8" s="27"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>20</v>
+        <v>110</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="E8" s="1" t="s">
         <v>7</v>
@@ -1191,15 +1213,15 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="E9" s="1" t="s">
         <v>7</v>
@@ -1213,23 +1235,23 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="30" t="s">
+      <c r="A10" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B10" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D10" s="2" t="s">
         <v>37</v>
       </c>
-      <c r="B10" s="2" t="s">
+      <c r="E10" s="2" t="s">
         <v>35</v>
       </c>
-      <c r="C10" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E10" s="2" t="s">
-        <v>36</v>
-      </c>
       <c r="F10" s="2" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="G10" s="2" t="b">
         <v>1</v>
@@ -1237,18 +1259,18 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
+      <c r="A11" s="28"/>
       <c r="B11" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D11" s="5" t="s">
         <v>53</v>
       </c>
-      <c r="C11" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D11" s="5" t="s">
+      <c r="E11" s="5" t="s">
         <v>54</v>
-      </c>
-      <c r="E11" s="5" t="s">
-        <v>55</v>
       </c>
       <c r="F11" s="5" t="s">
         <v>7</v>
@@ -1260,48 +1282,48 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A12" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>47</v>
+      </c>
+      <c r="C12" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D12" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="H12" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B12" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="H12" s="6" t="s">
-        <v>50</v>
-      </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="26" t="s">
+      <c r="A16" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B16" s="30"/>
+      <c r="C16" s="30"/>
+      <c r="D16" s="30"/>
+      <c r="E16" s="30"/>
+      <c r="F16" s="30"/>
+      <c r="G16" s="30"/>
+      <c r="H16" s="30"/>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A17" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B16" s="26"/>
-      <c r="C16" s="26"/>
-      <c r="D16" s="26"/>
-      <c r="E16" s="26"/>
-      <c r="F16" s="26"/>
-      <c r="G16" s="26"/>
-      <c r="H16" s="26"/>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="B17" s="33"/>
-      <c r="C17" s="33"/>
+      <c r="B17" s="29"/>
+      <c r="C17" s="29"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1354,7 +1376,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B7A7D7-7F99-4D47-A4D1-1272F654379A}">
-  <dimension ref="A1:H23"/>
+  <dimension ref="A1:H24"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -1363,7 +1385,7 @@
     <col min="4" max="4" width="73.83203125" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="19.4140625" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.25" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="79.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="89.5" style="1" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="49.25" style="1" bestFit="1" customWidth="1"/>
     <col min="9" max="16384" width="8.6640625" style="1"/>
   </cols>
@@ -1388,281 +1410,293 @@
         <v>17</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="30" t="s">
+      <c r="A2" s="34" t="s">
         <v>9</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C2" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D2" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="E2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G2" s="8" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3" s="35"/>
+      <c r="B3" s="1" t="s">
+        <v>106</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>103</v>
+      </c>
+      <c r="D3" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="E3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G3" s="25" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4" s="35"/>
+      <c r="B4" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="D4" s="1" t="s">
         <v>96</v>
       </c>
-      <c r="C2" s="34" t="s">
+      <c r="E4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G4" s="25"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5" s="35"/>
+      <c r="B5" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C5" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>100</v>
+      </c>
+      <c r="E5" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F5" s="1">
+        <v>0</v>
+      </c>
+      <c r="G5" s="25" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6" s="36"/>
+      <c r="B6" s="5" t="s">
+        <v>98</v>
+      </c>
+      <c r="C6" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D6" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F6" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G6" s="10" t="s">
+        <v>101</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7" s="26" t="s">
+        <v>11</v>
+      </c>
+      <c r="B7" s="2" t="s">
+        <v>2</v>
+      </c>
+      <c r="C7" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="D2" s="34" t="s">
-        <v>97</v>
-      </c>
-      <c r="E2" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="G2" s="8" t="s">
-        <v>106</v>
-      </c>
-    </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="31"/>
-      <c r="B3" s="34" t="s">
-        <v>98</v>
-      </c>
-      <c r="C3" s="34" t="s">
-        <v>40</v>
-      </c>
-      <c r="D3" s="34" t="s">
-        <v>99</v>
-      </c>
-      <c r="E3" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="F3" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="G3" s="25"/>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="31"/>
-      <c r="B4" s="34" t="s">
-        <v>100</v>
-      </c>
-      <c r="C4" s="34" t="s">
+      <c r="D7" s="2" t="s">
+        <v>24</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="F7" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="G7" s="8"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8" s="27"/>
+      <c r="B8" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>110</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="G8" s="25"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9" s="27"/>
+      <c r="B9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C9" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="D4" s="34" t="s">
-        <v>103</v>
-      </c>
-      <c r="E4" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="F4" s="34">
+      <c r="D9" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="1">
         <v>0</v>
       </c>
-      <c r="G4" s="25" t="s">
-        <v>105</v>
-      </c>
-    </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
-      <c r="B5" s="5" t="s">
-        <v>101</v>
-      </c>
-      <c r="C5" s="5" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="5" t="s">
-        <v>102</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F5" s="5" t="b">
+      <c r="G9" s="25" t="s">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="27"/>
+      <c r="B10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D10" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="1">
+        <v>0</v>
+      </c>
+      <c r="G10" s="25"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="27"/>
+      <c r="B11" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C11" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="E11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="F11" s="1" t="b">
         <v>1</v>
       </c>
-      <c r="G5" s="10" t="s">
-        <v>104</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="30" t="s">
-        <v>11</v>
-      </c>
-      <c r="B6" s="2" t="s">
-        <v>2</v>
-      </c>
-      <c r="C6" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="2" t="s">
-        <v>25</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="2" t="s">
+      <c r="G11" s="25"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12" s="26" t="s">
+        <v>36</v>
+      </c>
+      <c r="B12" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="D12" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" s="2" t="b">
+        <v>1</v>
+      </c>
+      <c r="G12" s="8"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13" s="28"/>
+      <c r="B13" s="5" t="s">
+        <v>52</v>
+      </c>
+      <c r="C13" s="5" t="s">
+        <v>21</v>
+      </c>
+      <c r="D13" s="5" t="s">
+        <v>53</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="5">
+        <v>0</v>
+      </c>
+      <c r="G13" s="10"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14" s="9" t="s">
+        <v>48</v>
+      </c>
+      <c r="B14" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="G6" s="8"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="31"/>
-      <c r="B7" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C7" s="1" t="s">
+      <c r="C14" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D7" s="1" t="s">
-        <v>33</v>
-      </c>
-      <c r="E7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="34" t="s">
-        <v>7</v>
-      </c>
-      <c r="G7" s="25"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="31"/>
-      <c r="B8" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C8" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="D8" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="E8" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F8" s="34">
-        <v>0</v>
-      </c>
-      <c r="G8" s="25" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="31"/>
-      <c r="B9" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C9" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="D9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="E9" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="34">
-        <v>0</v>
-      </c>
-      <c r="G9" s="25"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="31"/>
-      <c r="B10" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="C10" s="1" t="s">
-        <v>23</v>
-      </c>
-      <c r="D10" s="1" t="s">
-        <v>28</v>
-      </c>
-      <c r="E10" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="34" t="b">
-        <v>1</v>
-      </c>
-      <c r="G10" s="25"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="30" t="s">
-        <v>37</v>
-      </c>
-      <c r="B11" s="2" t="s">
-        <v>35</v>
-      </c>
-      <c r="C11" s="2" t="s">
-        <v>23</v>
-      </c>
-      <c r="D11" s="2" t="s">
-        <v>38</v>
-      </c>
-      <c r="E11" s="2" t="s">
-        <v>36</v>
-      </c>
-      <c r="F11" s="2" t="b">
-        <v>1</v>
-      </c>
-      <c r="G11" s="8"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="32"/>
-      <c r="B12" s="5" t="s">
-        <v>53</v>
-      </c>
-      <c r="C12" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D12" s="5" t="s">
-        <v>54</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F12" s="5">
-        <v>0</v>
-      </c>
-      <c r="G12" s="10"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="9" t="s">
+      <c r="D14" s="5" t="s">
+        <v>50</v>
+      </c>
+      <c r="E14" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F14" s="6" t="s">
+        <v>51</v>
+      </c>
+      <c r="G14" s="6" t="s">
         <v>49</v>
       </c>
-      <c r="B13" s="5" t="s">
-        <v>48</v>
-      </c>
-      <c r="C13" s="5" t="s">
-        <v>22</v>
-      </c>
-      <c r="D13" s="5" t="s">
-        <v>51</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="6" t="s">
-        <v>52</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="24" t="s">
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A18" s="24" t="s">
+        <v>81</v>
+      </c>
+      <c r="B18" s="24"/>
+      <c r="C18" s="24"/>
+      <c r="D18" s="24"/>
+      <c r="E18" s="24"/>
+      <c r="F18" s="24"/>
+      <c r="G18" s="24"/>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="29" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="24"/>
-      <c r="C17" s="24"/>
-      <c r="D17" s="24"/>
-      <c r="E17" s="24"/>
-      <c r="F17" s="24"/>
-      <c r="G17" s="24"/>
-    </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="33" t="s">
-        <v>83</v>
-      </c>
-      <c r="B18" s="33"/>
-      <c r="C18" s="33"/>
-      <c r="D18" s="11"/>
-      <c r="E18" s="11"/>
-      <c r="F18" s="11"/>
-      <c r="G18" s="11"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="11"/>
-      <c r="B19" s="11"/>
-      <c r="C19" s="11"/>
+      <c r="B19" s="29"/>
+      <c r="C19" s="29"/>
       <c r="D19" s="11"/>
       <c r="E19" s="11"/>
       <c r="F19" s="11"/>
@@ -1676,10 +1710,16 @@
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
-      <c r="H20" s="24"/>
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="H21" s="11"/>
+      <c r="A21" s="11"/>
+      <c r="B21" s="11"/>
+      <c r="C21" s="11"/>
+      <c r="D21" s="11"/>
+      <c r="E21" s="11"/>
+      <c r="F21" s="11"/>
+      <c r="G21" s="11"/>
+      <c r="H21" s="24"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H22" s="11"/>
@@ -1687,12 +1727,14 @@
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H23" s="11"/>
     </row>
+    <row r="24" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H24" s="11"/>
+    </row>
   </sheetData>
-  <mergeCells count="4">
-    <mergeCell ref="A2:A5"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A6:A10"/>
-    <mergeCell ref="A18:C18"/>
+  <mergeCells count="3">
+    <mergeCell ref="A12:A13"/>
+    <mergeCell ref="A7:A11"/>
+    <mergeCell ref="A19:C19"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1734,21 +1776,21 @@
         <v>17</v>
       </c>
       <c r="G1" s="8" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="27" t="s">
-        <v>87</v>
+      <c r="A2" s="31" t="s">
+        <v>86</v>
       </c>
       <c r="B2" s="12" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C2" s="13" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D2" s="13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E2" s="21" t="s">
         <v>7</v>
@@ -1759,15 +1801,15 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="28"/>
+      <c r="A3" s="32"/>
       <c r="B3" s="14" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C3" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D3" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E3" s="22" t="s">
         <v>7</v>
@@ -1776,19 +1818,19 @@
         <v>1</v>
       </c>
       <c r="G3" s="18" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
+      <c r="A4" s="32"/>
       <c r="B4" s="14" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C4" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D4" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="E4" s="22" t="s">
         <v>7</v>
@@ -1799,15 +1841,15 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="28"/>
+      <c r="A5" s="32"/>
       <c r="B5" s="14" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C5" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D5" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="E5" s="22" t="s">
         <v>7</v>
@@ -1818,15 +1860,15 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="28"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="14" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C6" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D6" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="E6" s="22" t="s">
         <v>7</v>
@@ -1837,15 +1879,15 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="28"/>
+      <c r="A7" s="32"/>
       <c r="B7" s="14" t="s">
+        <v>93</v>
+      </c>
+      <c r="C7" t="s">
+        <v>66</v>
+      </c>
+      <c r="D7" t="s">
         <v>94</v>
-      </c>
-      <c r="C7" t="s">
-        <v>67</v>
-      </c>
-      <c r="D7" t="s">
-        <v>95</v>
       </c>
       <c r="E7" s="22" t="s">
         <v>7</v>
@@ -1856,15 +1898,15 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="28"/>
+      <c r="A8" s="32"/>
       <c r="B8" s="14" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C8" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D8" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="E8" s="22" t="s">
         <v>7</v>
@@ -1875,57 +1917,57 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="28"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="14" t="s">
+        <v>62</v>
+      </c>
+      <c r="C9" t="s">
+        <v>67</v>
+      </c>
+      <c r="D9" t="s">
+        <v>76</v>
+      </c>
+      <c r="E9" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F9" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G9" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10" s="32"/>
+      <c r="B10" s="14" t="s">
+        <v>61</v>
+      </c>
+      <c r="C10" t="s">
+        <v>68</v>
+      </c>
+      <c r="D10" t="s">
+        <v>77</v>
+      </c>
+      <c r="E10" s="22" t="s">
+        <v>7</v>
+      </c>
+      <c r="F10" s="20" t="s">
+        <v>7</v>
+      </c>
+      <c r="G10" s="18" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11" s="32"/>
+      <c r="B11" s="14" t="s">
         <v>63</v>
       </c>
-      <c r="C9" t="s">
-        <v>68</v>
-      </c>
-      <c r="D9" t="s">
-        <v>77</v>
-      </c>
-      <c r="E9" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F9" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="G9" s="18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="28"/>
-      <c r="B10" s="14" t="s">
-        <v>62</v>
-      </c>
-      <c r="C10" t="s">
+      <c r="C11" t="s">
         <v>69</v>
       </c>
-      <c r="D10" t="s">
+      <c r="D11" t="s">
         <v>78</v>
-      </c>
-      <c r="E10" s="22" t="s">
-        <v>7</v>
-      </c>
-      <c r="F10" s="20" t="s">
-        <v>7</v>
-      </c>
-      <c r="G10" s="18" t="s">
-        <v>86</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
-      <c r="B11" s="14" t="s">
-        <v>64</v>
-      </c>
-      <c r="C11" t="s">
-        <v>70</v>
-      </c>
-      <c r="D11" t="s">
-        <v>79</v>
       </c>
       <c r="E11" s="22" t="s">
         <v>7</v>
@@ -1936,15 +1978,15 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="28"/>
+      <c r="A12" s="32"/>
       <c r="B12" s="14" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D12" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="E12" s="22" t="s">
         <v>7</v>
@@ -1955,15 +1997,15 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
+      <c r="A13" s="32"/>
       <c r="B13" s="14" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C13" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D13" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="E13" s="22" t="s">
         <v>7</v>
@@ -1974,15 +2016,15 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="28"/>
+      <c r="A14" s="32"/>
       <c r="B14" s="14" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C14" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D14" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E14" s="22" t="s">
         <v>7</v>
@@ -1993,15 +2035,15 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="29"/>
+      <c r="A15" s="33"/>
       <c r="B15" s="15" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C15" s="19" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D15" s="19" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="E15" s="23" t="s">
         <v>7</v>
@@ -2010,7 +2052,7 @@
         <v>0</v>
       </c>
       <c r="G15" s="16" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
@@ -2022,29 +2064,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="26" t="s">
-        <v>82</v>
-      </c>
-      <c r="B19" s="26"/>
-      <c r="C19" s="26"/>
-      <c r="D19" s="26"/>
-      <c r="E19" s="26"/>
-      <c r="F19" s="26"/>
-      <c r="G19" s="26"/>
+      <c r="A19" s="30" t="s">
+        <v>81</v>
+      </c>
+      <c r="B19" s="30"/>
+      <c r="C19" s="30"/>
+      <c r="D19" s="30"/>
+      <c r="E19" s="30"/>
+      <c r="F19" s="30"/>
+      <c r="G19" s="30"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="26" t="s">
-        <v>84</v>
-      </c>
-      <c r="B20" s="26"/>
-      <c r="C20" s="26"/>
+      <c r="A20" s="30" t="s">
+        <v>83</v>
+      </c>
+      <c r="B20" s="30"/>
+      <c r="C20" s="30"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="26" t="s">
-        <v>88</v>
-      </c>
-      <c r="B21" s="26"/>
-      <c r="C21" s="26"/>
+      <c r="A21" s="30" t="s">
+        <v>87</v>
+      </c>
+      <c r="B21" s="30"/>
+      <c r="C21" s="30"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>

<commit_message>
New property for BFW: TriggerOnUseOnContainer BFW now will trigger on use on projectile container depends on item settings
</commit_message>
<xml_diff>
--- a/English.xlsx
+++ b/English.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\SteamLibrary\steamapps\common\Barotrauma\LocalMods\Vanilla_Components_Expanded\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5B0C9189-882F-4FFA-A1A9-8B9389ADA110}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D587E7B-01B4-4442-98BC-1196C32F1812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="SwitchableRangedWeapon" sheetId="4" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="228" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="232" uniqueCount="114">
   <si>
     <t>switchableProjectiles</t>
     <phoneticPr fontId="1" type="noConversion"/>
@@ -459,6 +459,18 @@
   </si>
   <si>
     <t>An integer larger than 0</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>TriggerOnUseOnContainer</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>Whether the container of the projectile will be used during the firing process</t>
+    <phoneticPr fontId="1" type="noConversion"/>
+  </si>
+  <si>
+    <t>OnUse StatusEffects defined in the container will be triggered everytime the weapon shoots a projectile if true</t>
     <phoneticPr fontId="1" type="noConversion"/>
   </si>
 </sst>
@@ -634,7 +646,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="37">
+  <cellXfs count="35">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -695,6 +707,18 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -707,26 +731,8 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="12" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1049,7 +1055,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A2" s="26" t="s">
+      <c r="A2" s="30" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="2" t="s">
@@ -1075,7 +1081,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A3" s="27"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1" t="s">
         <v>38</v>
       </c>
@@ -1099,7 +1105,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A4" s="28"/>
+      <c r="A4" s="32"/>
       <c r="B4" s="1" t="s">
         <v>1</v>
       </c>
@@ -1121,7 +1127,7 @@
       <c r="H4" s="4"/>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A5" s="26" t="s">
+      <c r="A5" s="30" t="s">
         <v>11</v>
       </c>
       <c r="B5" s="2" t="s">
@@ -1145,7 +1151,7 @@
       <c r="H5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A6" s="27"/>
+      <c r="A6" s="31"/>
       <c r="B6" s="1" t="s">
         <v>3</v>
       </c>
@@ -1167,7 +1173,7 @@
       <c r="H6" s="4"/>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="27"/>
+      <c r="A7" s="31"/>
       <c r="B7" s="1" t="s">
         <v>4</v>
       </c>
@@ -1191,7 +1197,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A8" s="27"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1213,7 +1219,7 @@
       <c r="H8" s="4"/>
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A9" s="28"/>
+      <c r="A9" s="32"/>
       <c r="B9" s="1" t="s">
         <v>5</v>
       </c>
@@ -1235,7 +1241,7 @@
       <c r="H9" s="4"/>
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A10" s="26" t="s">
+      <c r="A10" s="30" t="s">
         <v>36</v>
       </c>
       <c r="B10" s="2" t="s">
@@ -1259,7 +1265,7 @@
       <c r="H10" s="8"/>
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A11" s="28"/>
+      <c r="A11" s="32"/>
       <c r="B11" s="5" t="s">
         <v>52</v>
       </c>
@@ -1307,23 +1313,23 @@
       </c>
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="B16" s="30"/>
-      <c r="C16" s="30"/>
-      <c r="D16" s="30"/>
-      <c r="E16" s="30"/>
-      <c r="F16" s="30"/>
-      <c r="G16" s="30"/>
-      <c r="H16" s="30"/>
+      <c r="B16" s="26"/>
+      <c r="C16" s="26"/>
+      <c r="D16" s="26"/>
+      <c r="E16" s="26"/>
+      <c r="F16" s="26"/>
+      <c r="G16" s="26"/>
+      <c r="H16" s="26"/>
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A17" s="29" t="s">
+      <c r="A17" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="B17" s="29"/>
-      <c r="C17" s="29"/>
+      <c r="B17" s="33"/>
+      <c r="C17" s="33"/>
       <c r="D17" s="11"/>
       <c r="E17" s="11"/>
       <c r="F17" s="11"/>
@@ -1376,7 +1382,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3B7A7D7-7F99-4D47-A4D1-1272F654379A}">
-  <dimension ref="A1:H24"/>
+  <dimension ref="A1:H25"/>
   <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" style="1" bestFit="1" customWidth="1"/>
@@ -1414,7 +1420,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="30" t="s">
         <v>9</v>
       </c>
       <c r="B2" s="1" t="s">
@@ -1437,7 +1443,7 @@
       </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="35"/>
+      <c r="A3" s="31"/>
       <c r="B3" s="1" t="s">
         <v>106</v>
       </c>
@@ -1458,7 +1464,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="35"/>
+      <c r="A4" s="31"/>
       <c r="B4" s="1" t="s">
         <v>95</v>
       </c>
@@ -1477,7 +1483,7 @@
       <c r="G4" s="25"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="35"/>
+      <c r="A5" s="31"/>
       <c r="B5" s="1" t="s">
         <v>97</v>
       </c>
@@ -1498,7 +1504,7 @@
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="36"/>
+      <c r="A6" s="32"/>
       <c r="B6" s="5" t="s">
         <v>98</v>
       </c>
@@ -1519,7 +1525,7 @@
       </c>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="26" t="s">
+      <c r="A7" s="30" t="s">
         <v>11</v>
       </c>
       <c r="B7" s="2" t="s">
@@ -1540,7 +1546,7 @@
       <c r="G7" s="8"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="27"/>
+      <c r="A8" s="31"/>
       <c r="B8" s="1" t="s">
         <v>3</v>
       </c>
@@ -1559,7 +1565,7 @@
       <c r="G8" s="25"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="27"/>
+      <c r="A9" s="31"/>
       <c r="B9" s="1" t="s">
         <v>4</v>
       </c>
@@ -1580,7 +1586,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="27"/>
+      <c r="A10" s="31"/>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
@@ -1599,7 +1605,7 @@
       <c r="G10" s="25"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="27"/>
+      <c r="A11" s="31"/>
       <c r="B11" s="1" t="s">
         <v>5</v>
       </c>
@@ -1618,7 +1624,7 @@
       <c r="G11" s="25"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="26" t="s">
+      <c r="A12" s="30" t="s">
         <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
@@ -1639,73 +1645,83 @@
       <c r="G12" s="8"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="28"/>
-      <c r="B13" s="5" t="s">
+      <c r="A13" s="31"/>
+      <c r="B13" s="34" t="s">
         <v>52</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="C13" s="34" t="s">
         <v>21</v>
       </c>
-      <c r="D13" s="5" t="s">
+      <c r="D13" s="34" t="s">
         <v>53</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F13" s="5">
+      <c r="E13" s="34" t="s">
+        <v>7</v>
+      </c>
+      <c r="F13" s="34">
         <v>0</v>
       </c>
-      <c r="G13" s="10"/>
+      <c r="G13" s="25"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="9" t="s">
+      <c r="A14" s="32"/>
+      <c r="B14" s="5" t="s">
+        <v>111</v>
+      </c>
+      <c r="C14" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="D14" s="5" t="s">
+        <v>112</v>
+      </c>
+      <c r="E14" s="5"/>
+      <c r="F14" s="5" t="b">
+        <v>1</v>
+      </c>
+      <c r="G14" s="10" t="s">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15" s="9" t="s">
         <v>48</v>
       </c>
-      <c r="B14" s="5" t="s">
+      <c r="B15" s="5" t="s">
         <v>47</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="C15" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="D14" s="5" t="s">
+      <c r="D15" s="5" t="s">
         <v>50</v>
       </c>
-      <c r="E14" s="5" t="s">
-        <v>7</v>
-      </c>
-      <c r="F14" s="6" t="s">
+      <c r="E15" s="5" t="s">
+        <v>7</v>
+      </c>
+      <c r="F15" s="6" t="s">
         <v>51</v>
       </c>
-      <c r="G14" s="6" t="s">
+      <c r="G15" s="6" t="s">
         <v>49</v>
       </c>
     </row>
-    <row r="18" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A18" s="24" t="s">
+    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A19" s="24" t="s">
         <v>81</v>
       </c>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
-      <c r="E18" s="24"/>
-      <c r="F18" s="24"/>
-      <c r="G18" s="24"/>
-    </row>
-    <row r="19" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A19" s="29" t="s">
+      <c r="B19" s="24"/>
+      <c r="C19" s="24"/>
+      <c r="D19" s="24"/>
+      <c r="E19" s="24"/>
+      <c r="F19" s="24"/>
+      <c r="G19" s="24"/>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="A20" s="33" t="s">
         <v>82</v>
       </c>
-      <c r="B19" s="29"/>
-      <c r="C19" s="29"/>
-      <c r="D19" s="11"/>
-      <c r="E19" s="11"/>
-      <c r="F19" s="11"/>
-      <c r="G19" s="11"/>
-    </row>
-    <row r="20" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A20" s="11"/>
-      <c r="B20" s="11"/>
-      <c r="C20" s="11"/>
+      <c r="B20" s="33"/>
+      <c r="C20" s="33"/>
       <c r="D20" s="11"/>
       <c r="E20" s="11"/>
       <c r="F20" s="11"/>
@@ -1719,10 +1735,16 @@
       <c r="E21" s="11"/>
       <c r="F21" s="11"/>
       <c r="G21" s="11"/>
-      <c r="H21" s="24"/>
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="H22" s="11"/>
+      <c r="A22" s="11"/>
+      <c r="B22" s="11"/>
+      <c r="C22" s="11"/>
+      <c r="D22" s="11"/>
+      <c r="E22" s="11"/>
+      <c r="F22" s="11"/>
+      <c r="G22" s="11"/>
+      <c r="H22" s="24"/>
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H23" s="11"/>
@@ -1730,11 +1752,15 @@
     <row r="24" spans="1:8" x14ac:dyDescent="0.3">
       <c r="H24" s="11"/>
     </row>
+    <row r="25" spans="1:8" x14ac:dyDescent="0.3">
+      <c r="H25" s="11"/>
+    </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A12:A13"/>
+  <mergeCells count="4">
     <mergeCell ref="A7:A11"/>
-    <mergeCell ref="A19:C19"/>
+    <mergeCell ref="A20:C20"/>
+    <mergeCell ref="A2:A6"/>
+    <mergeCell ref="A12:A14"/>
   </mergeCells>
   <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1780,7 +1806,7 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A2" s="31" t="s">
+      <c r="A2" s="27" t="s">
         <v>86</v>
       </c>
       <c r="B2" s="12" t="s">
@@ -1801,7 +1827,7 @@
       <c r="G2" s="17"/>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A3" s="32"/>
+      <c r="A3" s="28"/>
       <c r="B3" s="14" t="s">
         <v>56</v>
       </c>
@@ -1822,7 +1848,7 @@
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A4" s="32"/>
+      <c r="A4" s="28"/>
       <c r="B4" s="14" t="s">
         <v>57</v>
       </c>
@@ -1841,7 +1867,7 @@
       <c r="G4" s="18"/>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A5" s="32"/>
+      <c r="A5" s="28"/>
       <c r="B5" s="14" t="s">
         <v>58</v>
       </c>
@@ -1860,7 +1886,7 @@
       <c r="G5" s="18"/>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A6" s="32"/>
+      <c r="A6" s="28"/>
       <c r="B6" s="14" t="s">
         <v>60</v>
       </c>
@@ -1879,7 +1905,7 @@
       <c r="G6" s="18"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A7" s="32"/>
+      <c r="A7" s="28"/>
       <c r="B7" s="14" t="s">
         <v>93</v>
       </c>
@@ -1898,7 +1924,7 @@
       <c r="G7" s="18"/>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A8" s="32"/>
+      <c r="A8" s="28"/>
       <c r="B8" s="14" t="s">
         <v>59</v>
       </c>
@@ -1917,7 +1943,7 @@
       <c r="G8" s="18"/>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A9" s="32"/>
+      <c r="A9" s="28"/>
       <c r="B9" s="14" t="s">
         <v>62</v>
       </c>
@@ -1938,7 +1964,7 @@
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A10" s="32"/>
+      <c r="A10" s="28"/>
       <c r="B10" s="14" t="s">
         <v>61</v>
       </c>
@@ -1959,7 +1985,7 @@
       </c>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A11" s="32"/>
+      <c r="A11" s="28"/>
       <c r="B11" s="14" t="s">
         <v>63</v>
       </c>
@@ -1978,7 +2004,7 @@
       <c r="G11" s="18"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A12" s="32"/>
+      <c r="A12" s="28"/>
       <c r="B12" s="14" t="s">
         <v>64</v>
       </c>
@@ -1997,7 +2023,7 @@
       <c r="G12" s="18"/>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="32"/>
+      <c r="A13" s="28"/>
       <c r="B13" s="14" t="s">
         <v>65</v>
       </c>
@@ -2016,7 +2042,7 @@
       <c r="G13" s="18"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="32"/>
+      <c r="A14" s="28"/>
       <c r="B14" s="14" t="s">
         <v>88</v>
       </c>
@@ -2035,7 +2061,7 @@
       <c r="G14" s="18"/>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="33"/>
+      <c r="A15" s="29"/>
       <c r="B15" s="15" t="s">
         <v>89</v>
       </c>
@@ -2064,29 +2090,29 @@
       <c r="F17" s="1"/>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A19" s="30" t="s">
+      <c r="A19" s="26" t="s">
         <v>81</v>
       </c>
-      <c r="B19" s="30"/>
-      <c r="C19" s="30"/>
-      <c r="D19" s="30"/>
-      <c r="E19" s="30"/>
-      <c r="F19" s="30"/>
-      <c r="G19" s="30"/>
+      <c r="B19" s="26"/>
+      <c r="C19" s="26"/>
+      <c r="D19" s="26"/>
+      <c r="E19" s="26"/>
+      <c r="F19" s="26"/>
+      <c r="G19" s="26"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="26" t="s">
         <v>83</v>
       </c>
-      <c r="B20" s="30"/>
-      <c r="C20" s="30"/>
+      <c r="B20" s="26"/>
+      <c r="C20" s="26"/>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="26" t="s">
         <v>87</v>
       </c>
-      <c r="B21" s="30"/>
-      <c r="C21" s="30"/>
+      <c r="B21" s="26"/>
+      <c r="C21" s="26"/>
     </row>
   </sheetData>
   <mergeCells count="4">

</xml_diff>